<commit_message>
chore(daily-pickup): '우리팀' → 'GS' 라벨 전면 변경 (로직 불변)
- 요약/총평/주석/엑셀 개요의 '우리팀' 표기를 'GS'로 통일
- 세그 매핑·계산 로직은 현행 유지(OTA+G-OTA=GS, +홈페이지=FIT)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/july_pickup.xlsx
+++ b/docs/data/july_pickup.xlsx
@@ -782,7 +782,7 @@
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>- 기  준 : 전년 동기간 YOY  |  합계(FIT) = 우리팀(OTA+G-OTA) + 홈페이지(비관리)</t>
+          <t>- 기  준 : 전년 동기간 YOY  |  합계(FIT) = GS(OTA+G-OTA) + 홈페이지(비관리)</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>우리팀 (OTA+G-OTA)</t>
+          <t>GS (OTA+G-OTA)</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
@@ -1214,7 +1214,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>※ 투숙일 기준 30일 OTB · 홈페이지=자체채널(D멤버스·자사·FIT·제휴 등, 우리팀 비관리) · FIT=우리팀+홈페이지 · BSR(07/02)=소노 Booking Status Report FIT(전채널·시점차로 우리 FIT가 다소 낮음)</t>
+          <t>※ 투숙일 기준 30일 OTB · 홈페이지=자체채널(D멤버스·자사·FIT·제휴 등, GS 비관리) · FIT=GS+홈페이지 · BSR(07/02)=소노 Booking Status Report FIT(전채널·시점차로 우리 FIT가 다소 낮음)</t>
         </is>
       </c>
     </row>

</xml_diff>